<commit_message>
feat: initialize Shopify catalog migration framework
</commit_message>
<xml_diff>
--- a/02 Current Catalog/updated_products.xlsx
+++ b/02 Current Catalog/updated_products.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="R:\04 - National Accounts &amp; Pricing\07 - Website\01 - Website\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dschriver\Desktop\Claude CoWork\Projects\Shopify Catalog Update\02 Current Catalog\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6029C513-3B37-40A0-A0D0-2454020A0938}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F38AA9E6-ECCE-4202-ABC2-AF9C4653199B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{03105E7E-F27A-4740-B620-6F3A636340FA}"/>
+    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{03105E7E-F27A-4740-B620-6F3A636340FA}"/>
   </bookViews>
   <sheets>
     <sheet name="07.13.26" sheetId="3" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2004" uniqueCount="1840">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2004" uniqueCount="1842">
   <si>
     <t>DESCRIPTION</t>
   </si>
@@ -5579,6 +5579,12 @@
   </si>
   <si>
     <t>LIDS/CAPS - 4105-55</t>
+  </si>
+  <si>
+    <t>RAF032</t>
+  </si>
+  <si>
+    <t>MNR01</t>
   </si>
 </sst>
 </file>
@@ -5839,7 +5845,7 @@
         <name val="Manrope"/>
         <scheme val="none"/>
       </font>
-      <numFmt numFmtId="34" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
+      <numFmt numFmtId="164" formatCode="#,##0.00;\-#,##0.00"/>
     </dxf>
     <dxf>
       <font>
@@ -5857,7 +5863,7 @@
         <name val="Manrope"/>
         <scheme val="none"/>
       </font>
-      <numFmt numFmtId="164" formatCode="#,##0.00;\-#,##0.00"/>
+      <numFmt numFmtId="34" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
     </dxf>
     <dxf>
       <font>
@@ -5896,13 +5902,6 @@
       <numFmt numFmtId="30" formatCode="@"/>
     </dxf>
     <dxf>
-      <border outline="0">
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
       <border diagonalUp="0" diagonalDown="0">
         <left style="thin">
           <color indexed="64"/>
@@ -5934,6 +5933,13 @@
         <name val="Manrope"/>
         <scheme val="none"/>
       </font>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
     </dxf>
     <dxf>
       <font>
@@ -6067,15 +6073,15 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{91023302-41AC-41C5-9A8D-ED29A8306960}" name="Table44" displayName="Table44" ref="A8:D1125" totalsRowShown="0" headerRowDxfId="7" dataDxfId="6" headerRowBorderDxfId="4" tableBorderDxfId="5">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{91023302-41AC-41C5-9A8D-ED29A8306960}" name="Table44" displayName="Table44" ref="A8:D1125" totalsRowShown="0" headerRowDxfId="7" dataDxfId="5" headerRowBorderDxfId="6" tableBorderDxfId="4">
   <autoFilter ref="A8:D1125" xr:uid="{91023302-41AC-41C5-9A8D-ED29A8306960}"/>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{7723AEA6-5C28-47F7-8DFC-C878A9886384}" name="DESCRIPTION" dataDxfId="3"/>
     <tableColumn id="2" xr3:uid="{2424F045-A32A-4273-94BB-EF35C24439E2}" name="MPN" dataDxfId="2"/>
-    <tableColumn id="4" xr3:uid="{56FE45DD-D48C-40F4-BF4D-A51523B1C92B}" name="Column1" dataDxfId="0">
+    <tableColumn id="4" xr3:uid="{56FE45DD-D48C-40F4-BF4D-A51523B1C92B}" name="Column1" dataDxfId="1">
       <calculatedColumnFormula>D9*1.3</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{ED807D63-3B28-499F-AEC8-E946C5D2D96E}" name="PRICE" dataDxfId="1"/>
+    <tableColumn id="3" xr3:uid="{ED807D63-3B28-499F-AEC8-E946C5D2D96E}" name="PRICE" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -10821,7 +10827,7 @@
         <v>1697</v>
       </c>
       <c r="B302" s="14" t="s">
-        <v>1667</v>
+        <v>1840</v>
       </c>
       <c r="C302" s="21">
         <f t="shared" si="4"/>
@@ -16941,7 +16947,7 @@
         <v>789</v>
       </c>
       <c r="B710" s="14" t="s">
-        <v>763</v>
+        <v>1841</v>
       </c>
       <c r="C710" s="21">
         <f t="shared" si="10"/>
@@ -22747,7 +22753,7 @@
         <v>8132</v>
       </c>
       <c r="C1097" s="21">
-        <f t="shared" ref="C1097:C1160" si="17">D1097*1.3</f>
+        <f t="shared" ref="C1097:C1125" si="17">D1097*1.3</f>
         <v>32.487000000000002</v>
       </c>
       <c r="D1097" s="15">

</xml_diff>

<commit_message>
feat: add reusable Shopify import generation workflow
</commit_message>
<xml_diff>
--- a/02 Current Catalog/updated_products.xlsx
+++ b/02 Current Catalog/updated_products.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dschriver\Desktop\Claude CoWork\Projects\Shopify Catalog Update\02 Current Catalog\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F38AA9E6-ECCE-4202-ABC2-AF9C4653199B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B43EE243-1A83-4F54-8308-468BE412A2F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{03105E7E-F27A-4740-B620-6F3A636340FA}"/>
+    <workbookView xWindow="5910" yWindow="510" windowWidth="19680" windowHeight="13245" xr2:uid="{03105E7E-F27A-4740-B620-6F3A636340FA}"/>
   </bookViews>
   <sheets>
     <sheet name="07.13.26" sheetId="3" r:id="rId1"/>

</xml_diff>